<commit_message>
Daily dashboard refresh 2026-01-19 23:59
</commit_message>
<xml_diff>
--- a/data/FLM_Risk_Summary.xlsx
+++ b/data/FLM_Risk_Summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="31">
   <si>
     <t>Region</t>
   </si>
@@ -46,106 +46,67 @@
     <t>Makkah</t>
   </si>
   <si>
+    <t>Madinah</t>
+  </si>
+  <si>
+    <t>Taif</t>
+  </si>
+  <si>
+    <t>Jeddah</t>
+  </si>
+  <si>
     <t>Asir</t>
   </si>
   <si>
-    <t>Jeddah</t>
-  </si>
-  <si>
-    <t>Madinah</t>
-  </si>
-  <si>
-    <t>Taif</t>
-  </si>
-  <si>
     <t xml:space="preserve">Zaheer Ahmad Bashir Ahmad </t>
   </si>
   <si>
-    <t>Waqas Ahmad Nabi</t>
-  </si>
-  <si>
-    <t>Sohail Ahmed Muhammad Ahsan</t>
+    <t>Naseer Ahmed - Baboo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saleem Ullah Muhammad Nawaz </t>
+  </si>
+  <si>
+    <t>Faisal Javed Muhammed Javed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mohammed Hassan Ali Badrah </t>
+  </si>
+  <si>
+    <t>Raheel</t>
+  </si>
+  <si>
+    <t>Raed Ali Halabi</t>
+  </si>
+  <si>
+    <t>MUHAMMAD SHAFIQUE USMAN GHANI</t>
+  </si>
+  <si>
+    <t>Suliman Muhammad Idris</t>
   </si>
   <si>
     <t>Muhammad Umar Riaz Ahmed</t>
   </si>
   <si>
-    <t xml:space="preserve">Saleem Ullah Muhammad Nawaz </t>
-  </si>
-  <si>
     <t>Asif Taj</t>
   </si>
   <si>
-    <t xml:space="preserve">Mohammed Hassan Ali Badrah </t>
-  </si>
-  <si>
     <t>Rauf Azam Muhammad Azam</t>
   </si>
   <si>
-    <t>Naseer Ahmed - Baboo</t>
-  </si>
-  <si>
-    <t>Suliman Muhammad Idris</t>
-  </si>
-  <si>
-    <t>Faisal Javed Muhammed Javed</t>
+    <t>Abdulrahman Mohammed Yahya Mashraee</t>
   </si>
   <si>
     <t>Mohammad Akkas Ali Ayub Ali</t>
   </si>
   <si>
-    <t>Raed Ali Halabi</t>
-  </si>
-  <si>
-    <t>Wahid Ullah Sawal Faqir</t>
-  </si>
-  <si>
-    <t>Hasan Salem Omar Aldhaibani</t>
-  </si>
-  <si>
-    <t>Abdullah Gul Rahman</t>
-  </si>
-  <si>
-    <t>Syed Niaz Shah</t>
+    <t>Shabeer Muhammad Kunnumpurath</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khadim Hussain Muhammaed Alyas </t>
   </si>
   <si>
     <t>Hammad Hussain Muhammad iqbal</t>
-  </si>
-  <si>
-    <t>Raheel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muhammad Muzumail Khubaib </t>
-  </si>
-  <si>
-    <t>MUHAMMAD SHAFIQUE USMAN GHANI</t>
-  </si>
-  <si>
-    <t>Shabeer Muhammad Kunnumpurath</t>
-  </si>
-  <si>
-    <t>Bilal Muhammad Akbar</t>
-  </si>
-  <si>
-    <t>Faisal Atiah Salyazidi</t>
-  </si>
-  <si>
-    <t>Fayyaz Ali Ghulam Sarwar</t>
-  </si>
-  <si>
-    <t>Abdulrahman Mohammed Yahya Mashraee</t>
-  </si>
-  <si>
-    <t>Sohail Akhtar Syed Mohammed</t>
-  </si>
-  <si>
-    <t>Tabish Hasan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khadim Hussain Muhammaed Alyas </t>
-  </si>
-  <si>
-    <t>AzizUllah Mohammad</t>
   </si>
 </sst>
 </file>
@@ -503,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -540,39 +501,39 @@
         <v>14</v>
       </c>
       <c r="D2">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E2">
         <v>3</v>
       </c>
       <c r="F2">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G2">
-        <v>18.8</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
         <v>15</v>
       </c>
       <c r="D3">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G3">
-        <v>11.1</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -580,22 +541,22 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
       </c>
       <c r="D4">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="E4">
         <v>2</v>
       </c>
       <c r="F4">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="G4">
-        <v>10.5</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -603,22 +564,22 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
         <v>17</v>
       </c>
       <c r="D5">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="E5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="G5">
-        <v>7.8</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -626,45 +587,45 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
         <v>18</v>
       </c>
       <c r="D6">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="G6">
-        <v>7.3</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7" t="s">
         <v>19</v>
       </c>
       <c r="D7">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F7">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G7">
-        <v>7</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -678,16 +639,16 @@
         <v>20</v>
       </c>
       <c r="D8">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="E8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="G8">
-        <v>6.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -701,16 +662,16 @@
         <v>21</v>
       </c>
       <c r="D9">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="E9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="G9">
-        <v>6.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -718,22 +679,22 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C10" t="s">
         <v>22</v>
       </c>
       <c r="D10">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="G10">
-        <v>5.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -747,39 +708,39 @@
         <v>23</v>
       </c>
       <c r="D11">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F11">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="G11">
-        <v>4.8</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
         <v>24</v>
       </c>
       <c r="D12">
-        <v>87</v>
+        <v>34</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12">
-        <v>84</v>
+        <v>33</v>
       </c>
       <c r="G12">
-        <v>3.4</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -793,16 +754,16 @@
         <v>25</v>
       </c>
       <c r="D13">
-        <v>59</v>
+        <v>38</v>
       </c>
       <c r="E13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="G13">
-        <v>3.4</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -816,16 +777,16 @@
         <v>26</v>
       </c>
       <c r="D14">
-        <v>96</v>
+        <v>40</v>
       </c>
       <c r="E14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F14">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="G14">
-        <v>3.1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -839,16 +800,16 @@
         <v>27</v>
       </c>
       <c r="D15">
-        <v>65</v>
+        <v>43</v>
       </c>
       <c r="E15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="G15">
-        <v>3.1</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -862,16 +823,16 @@
         <v>28</v>
       </c>
       <c r="D16">
-        <v>32</v>
+        <v>123</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16">
-        <v>31</v>
+        <v>121</v>
       </c>
       <c r="G16">
-        <v>3.1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -879,344 +840,45 @@
         <v>7</v>
       </c>
       <c r="B17" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C17" t="s">
         <v>29</v>
       </c>
       <c r="D17">
-        <v>33</v>
+        <v>84</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="F17">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="G17">
-        <v>3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
         <v>30</v>
       </c>
       <c r="D18">
-        <v>70</v>
+        <v>109</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18">
-        <v>68</v>
+        <v>108</v>
       </c>
       <c r="G18">
-        <v>2.9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B19" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" t="s">
-        <v>31</v>
-      </c>
-      <c r="D19">
-        <v>142</v>
-      </c>
-      <c r="E19">
-        <v>4</v>
-      </c>
-      <c r="F19">
-        <v>138</v>
-      </c>
-      <c r="G19">
-        <v>2.8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" t="s">
-        <v>7</v>
-      </c>
-      <c r="B20" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20">
-        <v>41</v>
-      </c>
-      <c r="E20">
-        <v>1</v>
-      </c>
-      <c r="F20">
-        <v>40</v>
-      </c>
-      <c r="G20">
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" t="s">
-        <v>7</v>
-      </c>
-      <c r="B21" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D21">
-        <v>45</v>
-      </c>
-      <c r="E21">
-        <v>1</v>
-      </c>
-      <c r="F21">
-        <v>44</v>
-      </c>
-      <c r="G21">
-        <v>2.2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" t="s">
-        <v>7</v>
-      </c>
-      <c r="B22" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22">
-        <v>47</v>
-      </c>
-      <c r="E22">
-        <v>1</v>
-      </c>
-      <c r="F22">
-        <v>46</v>
-      </c>
-      <c r="G22">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" t="s">
-        <v>7</v>
-      </c>
-      <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" t="s">
-        <v>35</v>
-      </c>
-      <c r="D23">
-        <v>152</v>
-      </c>
-      <c r="E23">
-        <v>3</v>
-      </c>
-      <c r="F23">
-        <v>149</v>
-      </c>
-      <c r="G23">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" t="s">
-        <v>7</v>
-      </c>
-      <c r="B24" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" t="s">
-        <v>36</v>
-      </c>
-      <c r="D24">
-        <v>49</v>
-      </c>
-      <c r="E24">
-        <v>1</v>
-      </c>
-      <c r="F24">
-        <v>48</v>
-      </c>
-      <c r="G24">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" t="s">
-        <v>9</v>
-      </c>
-      <c r="C25" t="s">
-        <v>37</v>
-      </c>
-      <c r="D25">
-        <v>55</v>
-      </c>
-      <c r="E25">
-        <v>1</v>
-      </c>
-      <c r="F25">
-        <v>54</v>
-      </c>
-      <c r="G25">
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26" t="s">
-        <v>7</v>
-      </c>
-      <c r="B26" t="s">
-        <v>9</v>
-      </c>
-      <c r="C26" t="s">
-        <v>38</v>
-      </c>
-      <c r="D26">
-        <v>64</v>
-      </c>
-      <c r="E26">
-        <v>1</v>
-      </c>
-      <c r="F26">
-        <v>63</v>
-      </c>
-      <c r="G26">
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="A27" t="s">
-        <v>7</v>
-      </c>
-      <c r="B27" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D27">
-        <v>84</v>
-      </c>
-      <c r="E27">
-        <v>1</v>
-      </c>
-      <c r="F27">
-        <v>83</v>
-      </c>
-      <c r="G27">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28" t="s">
-        <v>7</v>
-      </c>
-      <c r="B28" t="s">
-        <v>9</v>
-      </c>
-      <c r="C28" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28">
-        <v>86</v>
-      </c>
-      <c r="E28">
-        <v>1</v>
-      </c>
-      <c r="F28">
-        <v>85</v>
-      </c>
-      <c r="G28">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" t="s">
-        <v>10</v>
-      </c>
-      <c r="C29" t="s">
-        <v>41</v>
-      </c>
-      <c r="D29">
-        <v>104</v>
-      </c>
-      <c r="E29">
-        <v>1</v>
-      </c>
-      <c r="F29">
-        <v>103</v>
-      </c>
-      <c r="G29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" t="s">
-        <v>7</v>
-      </c>
-      <c r="B30" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30" t="s">
-        <v>42</v>
-      </c>
-      <c r="D30">
-        <v>116</v>
-      </c>
-      <c r="E30">
-        <v>1</v>
-      </c>
-      <c r="F30">
-        <v>115</v>
-      </c>
-      <c r="G30">
         <v>0.9</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="A31" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31" t="s">
-        <v>10</v>
-      </c>
-      <c r="C31" t="s">
-        <v>43</v>
-      </c>
-      <c r="D31">
-        <v>132</v>
-      </c>
-      <c r="E31">
-        <v>1</v>
-      </c>
-      <c r="F31">
-        <v>131</v>
-      </c>
-      <c r="G31">
-        <v>0.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>